<commit_message>
up thay đổi kênh sóng
</commit_message>
<xml_diff>
--- a/tên và kênh sóng wifi các phòng.xlsx
+++ b/tên và kênh sóng wifi các phòng.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutoUpdateTV\MapDeviceNew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7ECE093-6292-41F0-AD62-922B17E02554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F487F823-DD78-4F6E-A5C9-2D9A0B970CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2329,7 +2329,7 @@
         <v>4</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D114" s="1"/>
       <c r="E114" s="2"/>

</xml_diff>

<commit_message>
up thay đổi kênh sóng1
</commit_message>
<xml_diff>
--- a/tên và kênh sóng wifi các phòng.xlsx
+++ b/tên và kênh sóng wifi các phòng.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutoUpdateTV\MapDeviceNew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BF8D64-0A27-4E73-9668-1742EE42F326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EA5A83D-6F81-4490-B363-100606797C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -1792,10 +1792,10 @@
         <v>77</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="2"/>

</xml_diff>